<commit_message>
Marcar en la planilla los municipios con borrador en Gmail
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JmGV4wYHZh4GQbMSRkNLeq
</commit_message>
<xml_diff>
--- a/data/municipalidades.xlsx
+++ b/data/municipalidades.xlsx
@@ -1002,6 +1002,11 @@
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Borrador creado en Gmail el 05-10-2026</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1322,6 +1327,11 @@
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Borrador creado en Gmail el 05-10-2026</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1557,6 +1567,11 @@
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Borrador creado en Gmail el 05-10-2026</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -17725,6 +17740,11 @@
       <c r="M317" t="inlineStr">
         <is>
           <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="P317" t="inlineStr">
+        <is>
+          <t>Borrador creado en Gmail el 05-10-2026</t>
         </is>
       </c>
     </row>
@@ -19307,7 +19327,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -19329,7 +19348,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>

</xml_diff>